<commit_message>
Upload chưa có alias lí do
</commit_message>
<xml_diff>
--- a/data/training/training_summary.xlsx
+++ b/data/training/training_summary.xlsx
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>107</v>
+        <v>898</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>182</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6">

</xml_diff>